<commit_message>
Removed extra samples before filtering
</commit_message>
<xml_diff>
--- a/meta/PUFFs_2025.xlsx
+++ b/meta/PUFFs_2025.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Passive air samplers" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="263">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -764,16 +764,7 @@
     <t xml:space="preserve">Method</t>
   </si>
   <si>
-    <t xml:space="preserve">Gromphadorhina portentosa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hissing cockroach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 minute walking each side of the PUF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caligo eurilachus</t>
+    <t xml:space="preserve">Caligo eurilochus</t>
   </si>
   <si>
     <t xml:space="preserve">Butterfly1</t>
@@ -2744,7 +2735,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.19"/>
@@ -2782,84 +2773,73 @@
         <v>250</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>253</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>255</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>257</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>261</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>263</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>